<commit_message>
split up data to be easily read per-sheet
</commit_message>
<xml_diff>
--- a/examples/universal_packed_bed_reactor/pump_rpm_vs_flow_rate_data/Pump Flow Rate Data.xlsx
+++ b/examples/universal_packed_bed_reactor/pump_rpm_vs_flow_rate_data/Pump Flow Rate Data.xlsx
@@ -1,35 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wille\Desktop\Projects-And-Code-Will-Martin\Excel Projects\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wille\Desktop\FVMFramework\examples\universal_packed_bed_reactor\pump_rpm_vs_flow_rate_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DAAF39E-CDDB-4DE5-8CDA-EDAA27BA39DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E43C867-F709-4160-BA7B-9C0572E0A5E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" xr2:uid="{61706984-1DB5-4F52-A4EA-C7FAFDCF8467}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{61706984-1DB5-4F52-A4EA-C7FAFDCF8467}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="data entry" sheetId="1" r:id="rId1"/>
+    <sheet name="10 RPM" sheetId="2" r:id="rId2"/>
+    <sheet name="5 RPM" sheetId="3" r:id="rId3"/>
+    <sheet name="1 RPM" sheetId="4" r:id="rId4"/>
+    <sheet name="0.3 RPM" sheetId="5" r:id="rId5"/>
+    <sheet name="50 RPM" sheetId="6" r:id="rId6"/>
+    <sheet name="25 RPM" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="2"/>
@@ -39,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="3">
   <si>
     <t xml:space="preserve">RPM </t>
   </si>
@@ -419,19 +414,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC1AD8B7-E345-42B9-91B1-9D43C9936D0B}">
-  <dimension ref="A2:R13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <dimension ref="B2:R13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="20.41796875" customWidth="1"/>
-    <col min="6" max="6" width="20.9453125" customWidth="1"/>
-    <col min="9" max="9" width="20.578125" customWidth="1"/>
-    <col min="12" max="12" width="21.3125" customWidth="1"/>
-    <col min="15" max="15" width="21.20703125" customWidth="1"/>
-    <col min="18" max="18" width="20.9453125" customWidth="1"/>
-    <col min="21" max="21" width="21.26171875" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" customWidth="1"/>
+    <col min="6" max="6" width="21" customWidth="1"/>
+    <col min="9" max="9" width="20.5703125" customWidth="1"/>
+    <col min="12" max="12" width="21.28515625" customWidth="1"/>
+    <col min="15" max="15" width="21.140625" customWidth="1"/>
+    <col min="18" max="18" width="21" customWidth="1"/>
+    <col min="21" max="21" width="21.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -469,7 +464,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>1</v>
       </c>
@@ -507,408 +502,992 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4">
-        <f>B4*60</f>
+    <row r="4" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B4">
         <v>30</v>
-      </c>
-      <c r="B4">
-        <v>0.5</v>
       </c>
       <c r="C4">
         <v>1.67</v>
       </c>
       <c r="E4">
-        <v>0.5</v>
+        <v>30</v>
       </c>
       <c r="F4">
         <v>0.86</v>
       </c>
       <c r="H4">
-        <v>0.5</v>
+        <v>30</v>
       </c>
       <c r="I4">
         <v>0.15</v>
       </c>
       <c r="K4">
-        <v>0.5</v>
+        <v>30</v>
       </c>
       <c r="L4">
         <v>0.09</v>
       </c>
       <c r="N4">
-        <v>0.5</v>
+        <v>30</v>
       </c>
       <c r="O4">
         <v>8.15</v>
       </c>
       <c r="Q4">
-        <v>0.5</v>
+        <v>30</v>
       </c>
       <c r="R4">
         <v>3.8</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5">
-        <f t="shared" ref="A5:A13" si="0">B5*60</f>
+    <row r="5" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B5">
         <v>60</v>
       </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
       <c r="E5">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="F5">
         <v>1.59</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="I5">
         <v>0.32</v>
       </c>
       <c r="K5">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="L5">
         <v>0.11</v>
       </c>
       <c r="N5">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="O5">
         <v>15.4</v>
       </c>
       <c r="Q5">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="R5">
         <v>7.7</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6">
-        <f t="shared" si="0"/>
+    <row r="6" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B6">
         <v>90</v>
-      </c>
-      <c r="B6">
-        <v>1.5</v>
       </c>
       <c r="C6">
         <v>4.67</v>
       </c>
       <c r="E6">
-        <v>1.5</v>
+        <v>90</v>
       </c>
       <c r="F6">
         <v>2.36</v>
       </c>
       <c r="H6">
-        <v>1.5</v>
+        <v>90</v>
       </c>
       <c r="I6">
         <v>0.46</v>
       </c>
       <c r="K6">
-        <v>1.5</v>
+        <v>90</v>
       </c>
       <c r="L6">
         <v>0.17</v>
       </c>
       <c r="N6">
-        <v>1.5</v>
+        <v>90</v>
       </c>
       <c r="O6">
         <v>23.3</v>
       </c>
       <c r="Q6">
-        <v>1.5</v>
+        <v>90</v>
       </c>
       <c r="R6">
         <v>11.4</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7">
-        <f t="shared" si="0"/>
+    <row r="7" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B7">
         <v>120</v>
-      </c>
-      <c r="B7">
-        <v>2</v>
       </c>
       <c r="C7">
         <v>6.19</v>
       </c>
       <c r="E7">
-        <v>2</v>
+        <v>120</v>
       </c>
       <c r="F7">
         <v>3.14</v>
       </c>
       <c r="H7">
-        <v>2</v>
+        <v>120</v>
       </c>
       <c r="I7">
         <v>0.62</v>
       </c>
       <c r="K7">
-        <v>2</v>
+        <v>120</v>
       </c>
       <c r="L7">
         <v>0.19</v>
       </c>
       <c r="N7">
-        <v>2</v>
+        <v>120</v>
       </c>
       <c r="O7">
         <v>30.8</v>
       </c>
       <c r="Q7">
-        <v>2</v>
+        <v>120</v>
       </c>
       <c r="R7">
         <v>15.3</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8">
-        <f t="shared" si="0"/>
+    <row r="8" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B8">
         <v>150</v>
-      </c>
-      <c r="B8">
-        <v>2.5</v>
       </c>
       <c r="C8">
         <v>7.9</v>
       </c>
       <c r="E8">
-        <v>2.5</v>
+        <v>150</v>
       </c>
       <c r="F8">
         <v>3.92</v>
       </c>
       <c r="H8">
-        <v>2.5</v>
+        <v>150</v>
       </c>
       <c r="I8">
         <v>0.77</v>
       </c>
       <c r="K8">
-        <v>2.5</v>
+        <v>150</v>
       </c>
       <c r="L8">
         <v>0.25</v>
       </c>
       <c r="N8">
-        <v>2.5</v>
+        <v>150</v>
       </c>
       <c r="Q8">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9">
-        <f t="shared" si="0"/>
+        <v>150</v>
+      </c>
+    </row>
+    <row r="9" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B9">
         <v>180</v>
-      </c>
-      <c r="B9">
-        <v>3</v>
       </c>
       <c r="C9">
         <v>9.3000000000000007</v>
       </c>
       <c r="E9">
-        <v>3</v>
+        <v>180</v>
       </c>
       <c r="F9">
         <v>4.6900000000000004</v>
       </c>
       <c r="H9">
-        <v>3</v>
+        <v>180</v>
       </c>
       <c r="I9">
         <v>0.94</v>
       </c>
       <c r="K9">
-        <v>3</v>
+        <v>180</v>
       </c>
       <c r="L9">
         <v>0.31</v>
       </c>
       <c r="N9">
-        <v>3</v>
+        <v>180</v>
       </c>
       <c r="O9">
         <v>46</v>
       </c>
       <c r="Q9">
-        <v>3</v>
+        <v>180</v>
       </c>
       <c r="R9">
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10">
-        <f t="shared" si="0"/>
+    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B10">
         <v>210</v>
-      </c>
-      <c r="B10">
-        <v>3.5</v>
       </c>
       <c r="C10">
         <v>10.88</v>
       </c>
       <c r="E10">
-        <v>3.5</v>
+        <v>210</v>
       </c>
       <c r="H10">
-        <v>3.5</v>
+        <v>210</v>
       </c>
       <c r="I10">
         <v>1.08</v>
       </c>
       <c r="K10">
-        <v>3.5</v>
+        <v>210</v>
       </c>
       <c r="L10">
         <v>0.36</v>
       </c>
       <c r="N10">
-        <v>3.5</v>
+        <v>210</v>
       </c>
       <c r="O10">
         <v>53.8</v>
       </c>
       <c r="Q10">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11">
-        <f t="shared" si="0"/>
+        <v>210</v>
+      </c>
+    </row>
+    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B11">
         <v>240</v>
-      </c>
-      <c r="B11">
-        <v>4</v>
       </c>
       <c r="C11">
         <v>12.43</v>
       </c>
       <c r="E11">
-        <v>4</v>
+        <v>240</v>
       </c>
       <c r="F11">
         <v>6.28</v>
       </c>
       <c r="H11">
-        <v>4</v>
+        <v>240</v>
       </c>
       <c r="I11">
         <v>1.25</v>
       </c>
       <c r="K11">
-        <v>4</v>
+        <v>240</v>
       </c>
       <c r="L11">
         <v>0.39</v>
       </c>
       <c r="N11">
-        <v>4</v>
+        <v>240</v>
       </c>
       <c r="O11">
         <v>61.4</v>
       </c>
       <c r="Q11">
-        <v>4</v>
+        <v>240</v>
       </c>
       <c r="R11">
         <v>30.65</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12">
-        <f t="shared" si="0"/>
+    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B12">
         <v>270</v>
-      </c>
-      <c r="B12">
-        <v>4.5</v>
       </c>
       <c r="C12">
         <v>14</v>
       </c>
       <c r="E12">
-        <v>4.5</v>
+        <v>270</v>
       </c>
       <c r="F12">
         <v>7.03</v>
       </c>
       <c r="H12">
-        <v>4.5</v>
+        <v>270</v>
       </c>
       <c r="I12">
         <v>1.4</v>
       </c>
       <c r="K12">
-        <v>4.5</v>
+        <v>270</v>
       </c>
       <c r="L12">
         <v>0.43</v>
       </c>
       <c r="N12">
-        <v>4.5</v>
+        <v>270</v>
       </c>
       <c r="O12">
         <v>69</v>
       </c>
       <c r="Q12">
-        <v>4.5</v>
+        <v>270</v>
       </c>
       <c r="R12">
         <v>34.6</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13">
-        <f t="shared" si="0"/>
+    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B13">
         <v>300</v>
-      </c>
-      <c r="B13">
-        <v>5</v>
       </c>
       <c r="C13">
         <v>15.49</v>
       </c>
       <c r="E13">
-        <v>5</v>
+        <v>300</v>
       </c>
       <c r="F13">
         <v>7.8</v>
       </c>
       <c r="H13">
-        <v>5</v>
+        <v>300</v>
       </c>
       <c r="I13">
         <v>1.56</v>
       </c>
       <c r="K13">
-        <v>5</v>
+        <v>300</v>
       </c>
       <c r="L13">
         <v>0.5</v>
       </c>
       <c r="N13">
-        <v>5</v>
+        <v>300</v>
       </c>
       <c r="O13">
         <v>76.599999999999994</v>
       </c>
       <c r="Q13">
+        <v>300</v>
+      </c>
+      <c r="R13">
+        <v>38.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D1F5EE8-A847-4344-BB22-B1C1A6F5B0F1}">
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>30</v>
+      </c>
+      <c r="B3">
+        <v>1.67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>90</v>
+      </c>
+      <c r="B5">
+        <v>4.67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>120</v>
+      </c>
+      <c r="B6">
+        <v>6.19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>150</v>
+      </c>
+      <c r="B7">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>180</v>
+      </c>
+      <c r="B8">
+        <v>9.3000000000000007</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>210</v>
+      </c>
+      <c r="B9">
+        <v>10.88</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>240</v>
+      </c>
+      <c r="B10">
+        <v>12.43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>270</v>
+      </c>
+      <c r="B11">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>300</v>
+      </c>
+      <c r="B12">
+        <v>15.49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E739598-CFB7-430D-9495-1877C379C766}">
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="9.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
         <v>5</v>
       </c>
-      <c r="R13">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>30</v>
+      </c>
+      <c r="B3">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>60</v>
+      </c>
+      <c r="B4">
+        <v>1.59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>90</v>
+      </c>
+      <c r="B5">
+        <v>2.36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>120</v>
+      </c>
+      <c r="B6">
+        <v>3.14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>150</v>
+      </c>
+      <c r="B7">
+        <v>3.92</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>180</v>
+      </c>
+      <c r="B8">
+        <v>4.6900000000000004</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>240</v>
+      </c>
+      <c r="B10">
+        <v>6.28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>270</v>
+      </c>
+      <c r="B11">
+        <v>7.03</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>300</v>
+      </c>
+      <c r="B12">
+        <v>7.8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5F07758-0EEA-4FD0-87B0-7CB4CC670E92}">
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>30</v>
+      </c>
+      <c r="B3">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>60</v>
+      </c>
+      <c r="B4">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>90</v>
+      </c>
+      <c r="B5">
+        <v>0.46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>120</v>
+      </c>
+      <c r="B6">
+        <v>0.62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>150</v>
+      </c>
+      <c r="B7">
+        <v>0.77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>180</v>
+      </c>
+      <c r="B8">
+        <v>0.94</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>210</v>
+      </c>
+      <c r="B9">
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>240</v>
+      </c>
+      <c r="B10">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>270</v>
+      </c>
+      <c r="B11">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>300</v>
+      </c>
+      <c r="B12">
+        <v>1.56</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{030129E0-78C9-41D9-B34E-9B8BDCFBDB0D}">
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>30</v>
+      </c>
+      <c r="B3">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>60</v>
+      </c>
+      <c r="B4">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>90</v>
+      </c>
+      <c r="B5">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>120</v>
+      </c>
+      <c r="B6">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>150</v>
+      </c>
+      <c r="B7">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>180</v>
+      </c>
+      <c r="B8">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>210</v>
+      </c>
+      <c r="B9">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>240</v>
+      </c>
+      <c r="B10">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>270</v>
+      </c>
+      <c r="B11">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>300</v>
+      </c>
+      <c r="B12">
+        <v>0.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEF69603-44D3-4BDD-BE26-FE11FE6877A1}">
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>30</v>
+      </c>
+      <c r="B3">
+        <v>8.15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>60</v>
+      </c>
+      <c r="B4">
+        <v>15.4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>90</v>
+      </c>
+      <c r="B5">
+        <v>23.3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>120</v>
+      </c>
+      <c r="B6">
+        <v>30.8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>180</v>
+      </c>
+      <c r="B8">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>210</v>
+      </c>
+      <c r="B9">
+        <v>53.8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>240</v>
+      </c>
+      <c r="B10">
+        <v>61.4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>270</v>
+      </c>
+      <c r="B11">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>300</v>
+      </c>
+      <c r="B12">
+        <v>76.599999999999994</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A2C20ED-79AC-4DFB-BDBB-60749915737A}">
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>30</v>
+      </c>
+      <c r="B3">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>60</v>
+      </c>
+      <c r="B4">
+        <v>7.7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>90</v>
+      </c>
+      <c r="B5">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>120</v>
+      </c>
+      <c r="B6">
+        <v>15.3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>180</v>
+      </c>
+      <c r="B8">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>240</v>
+      </c>
+      <c r="B10">
+        <v>30.65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>270</v>
+      </c>
+      <c r="B11">
+        <v>34.6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>300</v>
+      </c>
+      <c r="B12">
         <v>38.5</v>
       </c>
     </row>

</xml_diff>